<commit_message>
Updated Leaving Parental Home process -as it filters out students (those in cont.education), the LP process is now scheduled after Education Module in buildSchedule -removed the call from ageing() and scheduled it as its own Person.Processes.ConsiderLeavingHome event. -it now checks for age eligibility to be within [MIN_AGE_LEAVE_PH; MAX_AGE_ADULT_CHILD] -Removed the parent-availability test
</commit_message>
<xml_diff>
--- a/input/ES/parameters.xlsx
+++ b/input/ES/parameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsEU_AUG/input/ES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7445FB0E-5FA0-A34E-898B-C0933AED746A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F105DA-E651-3742-ABA9-6D61FB6AB4C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24440" yWindow="5440" windowWidth="20300" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="91">
   <si>
     <t>KEY</t>
   </si>
@@ -98,9 +98,6 @@
     <t>60</t>
   </si>
   <si>
-    <t>75</t>
-  </si>
-  <si>
     <t>TAXDB_REGIMES</t>
   </si>
   <si>
@@ -288,6 +285,15 @@
   </si>
   <si>
     <t>MAX_AGE_TO_STAY_IN_CONTINUOUS_EDUCATION</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>MIN_AGE_LEAVE_PH</t>
+  </si>
+  <si>
+    <t>MAX_AGE_ADULT_CHILD</t>
   </si>
 </sst>
 </file>
@@ -677,7 +683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="42.33203125" customWidth="1"/>
@@ -742,7 +748,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B8">
         <v>29</v>
@@ -825,7 +831,7 @@
         <v>19</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>25</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -854,7 +860,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B22" s="1">
         <v>6</v>
@@ -862,7 +868,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B23" s="1">
         <v>2011</v>
@@ -870,7 +876,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B24" s="1">
         <v>2020</v>
@@ -878,7 +884,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B25" s="1">
         <v>2019</v>
@@ -886,7 +892,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B26" s="1">
         <v>2019</v>
@@ -894,7 +900,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27" s="1">
         <v>0</v>
@@ -902,7 +908,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B28" s="1">
         <v>4000</v>
@@ -910,7 +916,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B29" s="1">
         <v>0</v>
@@ -918,7 +924,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B30" s="1">
         <v>15000</v>
@@ -926,7 +932,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B31" s="1">
         <v>14</v>
@@ -934,7 +940,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B32" s="1">
         <v>18</v>
@@ -942,7 +948,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B33" s="1">
         <v>49</v>
@@ -950,7 +956,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B34" s="1">
         <v>2015</v>
@@ -958,7 +964,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B35" s="1">
         <v>0.5</v>
@@ -966,7 +972,7 @@
     </row>
     <row r="36" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B36" s="2">
         <v>5.6000000000000001E-2</v>
@@ -974,7 +980,7 @@
     </row>
     <row r="37" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B37" s="10">
         <v>489</v>
@@ -982,7 +988,7 @@
     </row>
     <row r="38" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B38" s="10">
         <v>135</v>
@@ -990,7 +996,7 @@
     </row>
     <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B39" s="9">
         <v>45</v>
@@ -998,10 +1004,26 @@
     </row>
     <row r="40" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B40" s="9">
         <v>2018</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A41" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B41">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A42" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B42">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1021,7 +1043,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
@@ -1030,10 +1052,10 @@
     </row>
     <row r="3" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1041,7 +1063,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1049,7 +1071,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1057,7 +1079,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1065,7 +1087,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1073,7 +1095,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1081,7 +1103,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1089,7 +1111,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1097,7 +1119,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1105,7 +1127,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1113,7 +1135,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1121,7 +1143,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1129,7 +1151,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1137,7 +1159,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1145,7 +1167,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1153,7 +1175,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1161,7 +1183,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1169,7 +1191,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1177,7 +1199,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1185,7 +1207,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1193,7 +1215,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="17" x14ac:dyDescent="0.25">
@@ -1201,159 +1223,159 @@
         <v>22</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="17" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>